<commit_message>
scan: seg3 2026-06-17 19:29 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq4_2026-06-17.xlsx
+++ b/output/full_scan/batch_seq4_2026-06-17.xlsx
@@ -11191,7 +11191,7 @@
         <v/>
       </c>
       <c r="D203" s="2" t="n">
-        <v>249.2036228137918</v>
+        <v>249.2036228137917</v>
       </c>
       <c r="E203" s="2" t="n">
         <v>0</v>
@@ -11986,7 +11986,7 @@
         <v/>
       </c>
       <c r="D218" s="2" t="n">
-        <v>191.3174408974666</v>
+        <v>191.3174408974665</v>
       </c>
       <c r="E218" s="2" t="n">
         <v>21.75</v>

</xml_diff>